<commit_message>
feat: aplica retenção de 11 meses e otimiza pesquisa de preços
Exporta as datas de homologação e captura no Excel. Centraliza a janela de 11 meses, migra o esquema para 27 e aplica limpeza, compactação inicial e adequação de importações e sessões.

Pesquisa preços com unidade ou aproximação pelo índice dos itens e corrige a ordenação dos lotes por publicação. Inclui testes de regressão e medições em cópias isoladas.

Validação: compilação Release sem avisos ou erros e 478 testes aprovados.
</commit_message>
<xml_diff>
--- a/Planilha de Avaliação de Preços.xlsx
+++ b/Planilha de Avaliação de Preços.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PNCPKing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04D22D01-2C5C-4850-A823-DAD26A96A05A}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8415C350-45B0-494F-BD88-B9E22B6011B2}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>CNPJ</t>
-  </si>
-  <si>
-    <t>LINK PNCP</t>
   </si>
   <si>
     <t>VALOR DA COTAÇÃO</t>
@@ -95,9 +92,6 @@
     <t>{{ preco.cnpj }}</t>
   </si>
   <si>
-    <t>{{ link.pncp }}</t>
-  </si>
-  <si>
     <t>{{ preco.valor }}</t>
   </si>
   <si>
@@ -121,6 +115,12 @@
   <si>
     <t>{{ Inciso II se do PNCP e Inciso III se da internet }}</t>
   </si>
+  <si>
+    <t>{{ data.pncp }}</t>
+  </si>
+  <si>
+    <t>DATA HOMOLOGAÇÃO/OBTENÇÃO DOS PREÇOS</t>
+  </si>
 </sst>
 </file>
 
@@ -129,7 +129,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.0000;\-&quot;R$&quot;\ #,##0.0000"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -218,6 +218,13 @@
     </font>
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -588,9 +595,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -701,6 +705,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -999,7 +1006,7 @@
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
     <col min="2" max="2" width="76.85546875" customWidth="1"/>
     <col min="3" max="4" width="28.42578125" customWidth="1"/>
-    <col min="5" max="5" width="45.5703125" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" customWidth="1"/>
     <col min="6" max="6" width="20.28515625" customWidth="1"/>
     <col min="7" max="7" width="20" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="25.140625" hidden="1" customWidth="1"/>
@@ -1041,17 +1048,17 @@
     </row>
     <row r="2" spans="1:28" ht="180" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="42"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="41"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -1105,17 +1112,17 @@
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="45"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="43"/>
+      <c r="J4" s="44"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
@@ -1143,26 +1150,26 @@
       <c r="C5" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="38" t="s">
-        <v>19</v>
+      <c r="D5" s="37" t="s">
+        <v>17</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="G5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="H5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="J5" s="11" t="s">
         <v>9</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>10</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -1185,34 +1192,34 @@
     </row>
     <row r="6" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
-      <c r="B6" s="13" t="s">
-        <v>16</v>
+      <c r="B6" s="12" t="s">
+        <v>14</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="16" t="e">
+      <c r="G6" s="15" t="e">
         <f>IF(F6="","",SUM(AVERAGE(F7:F22)))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H6" s="17" t="e">
+      <c r="H6" s="16" t="e">
         <f t="shared" ref="H6:H22" si="0">(F6/G6)-1</f>
         <v>#VALUE!</v>
       </c>
-      <c r="I6" s="18" t="e">
+      <c r="I6" s="17" t="e">
         <f t="shared" ref="I6:I22" si="1">IF(G6="","",IF(H6&gt;0.25,"EXCESSIVO","VÁLIDO"))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J6" s="19" t="e">
+      <c r="J6" s="18" t="e">
         <f t="shared" ref="J6:J22" si="2">IF(G6="","",IF(H6&lt;-0.25,"INEXEQUÍVEL","VÁLIDO"))</f>
         <v>#DIV/0!</v>
       </c>
@@ -1240,28 +1247,28 @@
     </row>
     <row r="7" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16" t="str">
+      <c r="B7" s="19"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15" t="str">
         <f>IF(F7="","",SUM(AVERAGE(F6,F8:F22)))</f>
         <v/>
       </c>
-      <c r="H7" s="17" t="e">
+      <c r="H7" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I7" s="18" t="str">
+      <c r="I7" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J7" s="19" t="str">
+      <c r="J7" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1285,28 +1292,28 @@
     </row>
     <row r="8" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16" t="str">
+      <c r="B8" s="22"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15" t="str">
         <f>IF(F8="","",SUM(AVERAGE(F6:F7,F9:F22)))</f>
         <v/>
       </c>
-      <c r="H8" s="17" t="e">
+      <c r="H8" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I8" s="18" t="str">
+      <c r="I8" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J8" s="19" t="str">
+      <c r="J8" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1330,30 +1337,30 @@
     </row>
     <row r="9" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16" t="str">
+      <c r="B9" s="23"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15" t="str">
         <f>IF(F9="","",SUM(AVERAGE(F6:F8,F10:F22)))</f>
         <v/>
       </c>
-      <c r="H9" s="17" t="e">
+      <c r="H9" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I9" s="18" t="str">
+      <c r="I9" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J9" s="19" t="str">
+      <c r="J9" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K9" s="22">
+      <c r="K9" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1377,30 +1384,30 @@
     </row>
     <row r="10" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16" t="str">
+      <c r="B10" s="23"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15" t="str">
         <f>IF(F10="","",SUM(AVERAGE(F6:F9,F11:F22)))</f>
         <v/>
       </c>
-      <c r="H10" s="17" t="e">
+      <c r="H10" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I10" s="18" t="str">
+      <c r="I10" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J10" s="19" t="str">
+      <c r="J10" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K10" s="22">
+      <c r="K10" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1424,30 +1431,30 @@
     </row>
     <row r="11" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B11" s="24"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16" t="str">
+      <c r="B11" s="23"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15" t="str">
         <f>IF(F11="","",SUM(AVERAGE(F6:F10,F12:F22)))</f>
         <v/>
       </c>
-      <c r="H11" s="17" t="e">
+      <c r="H11" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I11" s="18" t="str">
+      <c r="I11" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J11" s="19" t="str">
+      <c r="J11" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K11" s="22">
+      <c r="K11" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1471,30 +1478,30 @@
     </row>
     <row r="12" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16" t="str">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15" t="str">
         <f>IF(F12="","",SUM(AVERAGE(F6:F11,F13:F22)))</f>
         <v/>
       </c>
-      <c r="H12" s="17" t="e">
+      <c r="H12" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I12" s="18" t="str">
+      <c r="I12" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J12" s="19" t="str">
+      <c r="J12" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1518,30 +1525,30 @@
     </row>
     <row r="13" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16" t="str">
+      <c r="B13" s="23"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15" t="str">
         <f>IF(F13="","",SUM(AVERAGE(F6:F12,F14:F22)))</f>
         <v/>
       </c>
-      <c r="H13" s="17" t="e">
+      <c r="H13" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I13" s="18" t="str">
+      <c r="I13" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J13" s="19" t="str">
+      <c r="J13" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K13" s="22">
+      <c r="K13" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1565,30 +1572,30 @@
     </row>
     <row r="14" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16" t="str">
+      <c r="B14" s="23"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15" t="str">
         <f>IF(F14="","",SUM(AVERAGE(F6:F13,F15:F22)))</f>
         <v/>
       </c>
-      <c r="H14" s="17" t="e">
+      <c r="H14" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I14" s="18" t="str">
+      <c r="I14" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J14" s="19" t="str">
+      <c r="J14" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K14" s="22">
+      <c r="K14" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1612,30 +1619,30 @@
     </row>
     <row r="15" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16" t="str">
+      <c r="B15" s="24"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15" t="str">
         <f>IF(F15="","",SUM(AVERAGE(F6:F14,F16:F22)))</f>
         <v/>
       </c>
-      <c r="H15" s="17" t="e">
+      <c r="H15" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I15" s="18" t="str">
+      <c r="I15" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J15" s="19" t="str">
+      <c r="J15" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K15" s="22">
+      <c r="K15" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1659,30 +1666,30 @@
     </row>
     <row r="16" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16" t="str">
+      <c r="B16" s="25"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15" t="str">
         <f>IF(F16="","",SUM(AVERAGE(F6:F15,F17:F22)))</f>
         <v/>
       </c>
-      <c r="H16" s="17" t="e">
+      <c r="H16" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I16" s="18" t="str">
+      <c r="I16" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J16" s="19" t="str">
+      <c r="J16" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K16" s="22">
+      <c r="K16" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1706,30 +1713,30 @@
     </row>
     <row r="17" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B17" s="27"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16" t="str">
+      <c r="B17" s="26"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15" t="str">
         <f>IF(F17="","",SUM(AVERAGE(F6:F16,F18:F22)))</f>
         <v/>
       </c>
-      <c r="H17" s="17" t="e">
+      <c r="H17" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I17" s="18" t="str">
+      <c r="I17" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J17" s="19" t="str">
+      <c r="J17" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K17" s="22">
+      <c r="K17" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1753,30 +1760,30 @@
     </row>
     <row r="18" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B18" s="27"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16" t="str">
+      <c r="B18" s="26"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15" t="str">
         <f>IF(F18="","",SUM(AVERAGE(F6:F17,F19:F22)))</f>
         <v/>
       </c>
-      <c r="H18" s="17" t="e">
+      <c r="H18" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I18" s="18" t="str">
+      <c r="I18" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J18" s="19" t="str">
+      <c r="J18" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K18" s="22">
+      <c r="K18" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1800,30 +1807,30 @@
     </row>
     <row r="19" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16" t="str">
+      <c r="B19" s="26"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15" t="str">
         <f>IF(F19="","",SUM(AVERAGE(F6:F18,F20:F22)))</f>
         <v/>
       </c>
-      <c r="H19" s="17" t="e">
+      <c r="H19" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I19" s="18" t="str">
+      <c r="I19" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J19" s="19" t="str">
+      <c r="J19" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K19" s="22">
+      <c r="K19" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1847,30 +1854,30 @@
     </row>
     <row r="20" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16" t="str">
+      <c r="B20" s="26"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15" t="str">
         <f>IF(F20="","",SUM(AVERAGE(F6:F19,F21:F22)))</f>
         <v/>
       </c>
-      <c r="H20" s="17" t="e">
+      <c r="H20" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I20" s="18" t="str">
+      <c r="I20" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J20" s="19" t="str">
+      <c r="J20" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K20" s="22">
+      <c r="K20" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1894,30 +1901,30 @@
     </row>
     <row r="21" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B21" s="27"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16" t="str">
+      <c r="B21" s="26"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15" t="str">
         <f>IF(F21="","",SUM(AVERAGE(F6:F20,F22)))</f>
         <v/>
       </c>
-      <c r="H21" s="17" t="e">
+      <c r="H21" s="16" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I21" s="18" t="str">
+      <c r="I21" s="17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J21" s="19" t="str">
+      <c r="J21" s="18" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K21" s="22">
+      <c r="K21" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1941,30 +1948,30 @@
     </row>
     <row r="22" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30" t="str">
+      <c r="B22" s="27"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29" t="str">
         <f>IF(F22="","",SUM(AVERAGE(F6:F21)))</f>
         <v/>
       </c>
-      <c r="H22" s="31" t="e">
+      <c r="H22" s="30" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="I22" s="32" t="str">
+      <c r="I22" s="31" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="J22" s="33" t="str">
+      <c r="J22" s="32" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K22" s="22">
+      <c r="K22" s="21">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1988,16 +1995,16 @@
     </row>
     <row r="23" spans="1:28" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
-      <c r="B23" s="34" t="s">
-        <v>15</v>
+      <c r="B23" s="33" t="s">
+        <v>13</v>
       </c>
-      <c r="C23" s="46" t="e">
+      <c r="C23" s="45" t="e">
         <f>IF(F6="","",SUM(K6:K22)/COUNTIF(K6:K22,"&gt;0"))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D23" s="47"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="49"/>
+      <c r="D23" s="46"/>
+      <c r="E23" s="47"/>
+      <c r="F23" s="48"/>
       <c r="G23" s="4"/>
       <c r="H23" s="5"/>
       <c r="I23" s="6"/>
@@ -2054,37 +2061,37 @@
       <c r="AB24" s="2"/>
     </row>
     <row r="25" spans="1:28" ht="77.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="35"/>
-      <c r="B25" s="36" t="s">
-        <v>17</v>
+      <c r="A25" s="34"/>
+      <c r="B25" s="35" t="s">
+        <v>15</v>
       </c>
-      <c r="C25" s="50" t="s">
-        <v>18</v>
+      <c r="C25" s="49" t="s">
+        <v>16</v>
       </c>
-      <c r="D25" s="51"/>
-      <c r="E25" s="51"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="51"/>
-      <c r="H25" s="51"/>
-      <c r="I25" s="52"/>
-      <c r="J25" s="37"/>
-      <c r="K25" s="37"/>
-      <c r="L25" s="37"/>
-      <c r="M25" s="37"/>
-      <c r="N25" s="37"/>
-      <c r="O25" s="37"/>
-      <c r="P25" s="37"/>
-      <c r="Q25" s="37"/>
-      <c r="R25" s="37"/>
-      <c r="S25" s="37"/>
-      <c r="T25" s="37"/>
-      <c r="U25" s="37"/>
-      <c r="V25" s="37"/>
-      <c r="W25" s="37"/>
-      <c r="X25" s="37"/>
-      <c r="Y25" s="37"/>
-      <c r="Z25" s="37"/>
-      <c r="AA25" s="37"/>
+      <c r="D25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="50"/>
+      <c r="G25" s="50"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="51"/>
+      <c r="J25" s="36"/>
+      <c r="K25" s="36"/>
+      <c r="L25" s="36"/>
+      <c r="M25" s="36"/>
+      <c r="N25" s="36"/>
+      <c r="O25" s="36"/>
+      <c r="P25" s="36"/>
+      <c r="Q25" s="36"/>
+      <c r="R25" s="36"/>
+      <c r="S25" s="36"/>
+      <c r="T25" s="36"/>
+      <c r="U25" s="36"/>
+      <c r="V25" s="36"/>
+      <c r="W25" s="36"/>
+      <c r="X25" s="36"/>
+      <c r="Y25" s="36"/>
+      <c r="Z25" s="36"/>
+      <c r="AA25" s="36"/>
       <c r="AB25" s="2"/>
     </row>
     <row r="26" spans="1:28" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">

</xml_diff>